<commit_message>
scan: seg6 2026-07-15 19:02 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq7_2026-07-15.xlsx
+++ b/output/full_scan/batch_seq7_2026-07-15.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O127"/>
+  <dimension ref="A1:O128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4078,21 +4078,21 @@
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
-        <v>6835</v>
+        <v>6831</v>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>圓裕</t>
+          <t>邁科</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
         <v/>
       </c>
       <c r="D69" s="2" t="n">
-        <v>327.8997052119791</v>
+        <v>328.5848632975021</v>
       </c>
       <c r="E69" s="2" t="n">
-        <v>32.95</v>
+        <v>710</v>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
@@ -4103,13 +4103,13 @@
         <v>0</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>27.31389067544913</v>
+        <v>43.2811478945184</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>30.71454947071413</v>
+        <v>23.3178036024913</v>
       </c>
       <c r="J69" s="2" t="n">
-        <v>1.60774928378941</v>
+        <v>0.2552706241418368</v>
       </c>
       <c r="K69" s="2" t="n">
         <v>0</v>
@@ -4121,31 +4121,31 @@
         <v>-1</v>
       </c>
       <c r="N69" s="2" t="n">
-        <v>-0.1719365658875357</v>
+        <v>-24.71566044708021</v>
       </c>
       <c r="O69" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
-        <v>6742</v>
+        <v>6835</v>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>澤米</t>
+          <t>圓裕</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
         <v/>
       </c>
       <c r="D70" s="2" t="n">
-        <v>319.3516247550556</v>
+        <v>327.8997052119791</v>
       </c>
       <c r="E70" s="2" t="n">
-        <v>51.7</v>
+        <v>32.95</v>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
@@ -4156,13 +4156,13 @@
         <v>0</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>34.95598878495284</v>
+        <v>27.31389067544913</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>23.64700177173711</v>
+        <v>30.71454947071413</v>
       </c>
       <c r="J70" s="2" t="n">
-        <v>0.1586246260899506</v>
+        <v>1.60774928378941</v>
       </c>
       <c r="K70" s="2" t="n">
         <v>0</v>
@@ -4174,31 +4174,31 @@
         <v>-1</v>
       </c>
       <c r="N70" s="2" t="n">
-        <v>-2.159862184463309</v>
+        <v>-0.1719365658875357</v>
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>volume_break, market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
-        <v>6664</v>
+        <v>6742</v>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>群翊</t>
+          <t>澤米</t>
         </is>
       </c>
       <c r="C71" s="2" t="n">
         <v/>
       </c>
       <c r="D71" s="2" t="n">
-        <v>313.7742194864342</v>
+        <v>319.3516247550556</v>
       </c>
       <c r="E71" s="2" t="n">
-        <v>394.5</v>
+        <v>51.7</v>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
@@ -4209,16 +4209,16 @@
         <v>0</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>52.10027798430875</v>
+        <v>34.95598878495284</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>18.29448581854033</v>
+        <v>23.64700177173711</v>
       </c>
       <c r="J71" s="2" t="n">
-        <v>0.8542678651391941</v>
+        <v>0.1586246260899506</v>
       </c>
       <c r="K71" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L71" s="2" t="n">
         <v>0</v>
@@ -4227,31 +4227,31 @@
         <v>-1</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>1.708125547175436</v>
+        <v>-2.159862184463309</v>
       </c>
       <c r="O71" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
-        <v>6570</v>
+        <v>6664</v>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>維田</t>
+          <t>群翊</t>
         </is>
       </c>
       <c r="C72" s="2" t="n">
         <v/>
       </c>
       <c r="D72" s="2" t="n">
-        <v>308.0421301747058</v>
+        <v>313.7742194864342</v>
       </c>
       <c r="E72" s="2" t="n">
-        <v>49.9</v>
+        <v>394.5</v>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
@@ -4262,16 +4262,16 @@
         <v>0</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>43.52702506965062</v>
+        <v>52.10027798430875</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>19.96624547058188</v>
+        <v>18.29448581854033</v>
       </c>
       <c r="J72" s="2" t="n">
-        <v>0.9125662585371844</v>
+        <v>0.8542678651391941</v>
       </c>
       <c r="K72" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L72" s="2" t="n">
         <v>0</v>
@@ -4280,31 +4280,31 @@
         <v>-1</v>
       </c>
       <c r="N72" s="2" t="n">
-        <v>-0.4970246860242759</v>
+        <v>1.708125547175436</v>
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, kd_golden_cross, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
-        <v>6840</v>
+        <v>6570</v>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>東研信超</t>
+          <t>維田</t>
         </is>
       </c>
       <c r="C73" s="2" t="n">
         <v/>
       </c>
       <c r="D73" s="2" t="n">
-        <v>305.0053921471465</v>
+        <v>308.0421301747058</v>
       </c>
       <c r="E73" s="2" t="n">
-        <v>62.5</v>
+        <v>49.9</v>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
@@ -4315,16 +4315,16 @@
         <v>0</v>
       </c>
       <c r="H73" s="2" t="n">
-        <v>44.44372952506817</v>
+        <v>43.52702506965062</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>11.41935497791801</v>
+        <v>19.96624547058188</v>
       </c>
       <c r="J73" s="2" t="n">
-        <v>0.6085367724403927</v>
+        <v>0.9125662585371844</v>
       </c>
       <c r="K73" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L73" s="2" t="n">
         <v>0</v>
@@ -4333,7 +4333,7 @@
         <v>-1</v>
       </c>
       <c r="N73" s="2" t="n">
-        <v>-0.2048568594289759</v>
+        <v>-0.4970246860242759</v>
       </c>
       <c r="O73" s="2" t="inlineStr">
         <is>
@@ -4343,21 +4343,21 @@
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
-        <v>6679</v>
+        <v>6840</v>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>鈺太</t>
+          <t>東研信超</t>
         </is>
       </c>
       <c r="C74" s="2" t="n">
         <v/>
       </c>
       <c r="D74" s="2" t="n">
-        <v>303.4228410445121</v>
+        <v>305.0053921471465</v>
       </c>
       <c r="E74" s="2" t="n">
-        <v>243</v>
+        <v>62.5</v>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
@@ -4368,16 +4368,16 @@
         <v>0</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>36.11398211840342</v>
+        <v>44.44372952506817</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>24.19556329792537</v>
+        <v>11.41935497791801</v>
       </c>
       <c r="J74" s="2" t="n">
-        <v>0.5843269324742805</v>
+        <v>0.6085367724403927</v>
       </c>
       <c r="K74" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L74" s="2" t="n">
         <v>0</v>
@@ -4386,31 +4386,31 @@
         <v>-1</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>-2.29489783331308</v>
+        <v>-0.2048568594289759</v>
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, kd_golden_cross, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
-        <v>6584</v>
+        <v>6679</v>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>南俊國際</t>
+          <t>鈺太</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
         <v/>
       </c>
       <c r="D75" s="2" t="n">
-        <v>302.8258803306682</v>
+        <v>303.4228410445121</v>
       </c>
       <c r="E75" s="2" t="n">
-        <v>666</v>
+        <v>243</v>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
@@ -4421,13 +4421,13 @@
         <v>0</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>48.91380212788646</v>
+        <v>36.11398211840342</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>11.18503551487324</v>
+        <v>24.19556329792537</v>
       </c>
       <c r="J75" s="2" t="n">
-        <v>0.3027923182656233</v>
+        <v>0.5843269324742805</v>
       </c>
       <c r="K75" s="2" t="n">
         <v>0</v>
@@ -4439,31 +4439,31 @@
         <v>-1</v>
       </c>
       <c r="N75" s="2" t="n">
-        <v>-3.526470350307084</v>
+        <v>-2.29489783331308</v>
       </c>
       <c r="O75" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
-        <v>6781</v>
+        <v>6584</v>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>AES-KY</t>
+          <t>南俊國際</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
         <v/>
       </c>
       <c r="D76" s="2" t="n">
-        <v>302.606201573097</v>
+        <v>302.8258803306682</v>
       </c>
       <c r="E76" s="2" t="n">
-        <v>1040</v>
+        <v>666</v>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
@@ -4474,13 +4474,13 @@
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>37.50284443620395</v>
+        <v>48.91380212788646</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>12.3731503104857</v>
+        <v>11.18503551487324</v>
       </c>
       <c r="J76" s="2" t="n">
-        <v>0.6973438859994946</v>
+        <v>0.3027923182656233</v>
       </c>
       <c r="K76" s="2" t="n">
         <v>0</v>
@@ -4492,31 +4492,31 @@
         <v>-1</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>-15.92864713781622</v>
+        <v>-3.526470350307084</v>
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
-        <v>6588</v>
+        <v>6781</v>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>東典光電</t>
+          <t>AES-KY</t>
         </is>
       </c>
       <c r="C77" s="2" t="n">
         <v/>
       </c>
       <c r="D77" s="2" t="n">
-        <v>299.153291613521</v>
+        <v>302.606201573097</v>
       </c>
       <c r="E77" s="2" t="n">
-        <v>80.7</v>
+        <v>1040</v>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
@@ -4527,13 +4527,13 @@
         <v>0</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>34.06322610033682</v>
+        <v>37.50284443620395</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>24.07220434424154</v>
+        <v>12.3731503104857</v>
       </c>
       <c r="J77" s="2" t="n">
-        <v>0.910213278497658</v>
+        <v>0.6973438859994946</v>
       </c>
       <c r="K77" s="2" t="n">
         <v>0</v>
@@ -4545,31 +4545,31 @@
         <v>-1</v>
       </c>
       <c r="N77" s="2" t="n">
-        <v>-0.1782595997192082</v>
+        <v>-15.92864713781622</v>
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
-        <v>6735</v>
+        <v>6588</v>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>美達科技</t>
+          <t>東典光電</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
         <v/>
       </c>
       <c r="D78" s="2" t="n">
-        <v>297.9788889286131</v>
+        <v>299.153291613521</v>
       </c>
       <c r="E78" s="2" t="n">
-        <v>75.3</v>
+        <v>80.7</v>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
@@ -4580,16 +4580,16 @@
         <v>0</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>28.60871854513493</v>
+        <v>34.06322610033682</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>15.13048968251978</v>
+        <v>24.07220434424154</v>
       </c>
       <c r="J78" s="2" t="n">
-        <v>0.4485589291592267</v>
+        <v>0.910213278497658</v>
       </c>
       <c r="K78" s="2" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="L78" s="2" t="n">
         <v>0</v>
@@ -4598,31 +4598,31 @@
         <v>-1</v>
       </c>
       <c r="N78" s="2" t="n">
-        <v>-0.8446889772863546</v>
+        <v>-0.1782595997192082</v>
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, foreign_buy_3d</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
-        <v>6768</v>
+        <v>6735</v>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>志強-KY</t>
+          <t>美達科技</t>
         </is>
       </c>
       <c r="C79" s="2" t="n">
         <v/>
       </c>
       <c r="D79" s="2" t="n">
-        <v>296.8022212840239</v>
+        <v>297.9788889286131</v>
       </c>
       <c r="E79" s="2" t="n">
-        <v>71</v>
+        <v>75.3</v>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
@@ -4633,16 +4633,16 @@
         <v>0</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>28.31496916822526</v>
+        <v>28.60871854513493</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>31.18468131202025</v>
+        <v>15.13048968251978</v>
       </c>
       <c r="J79" s="2" t="n">
-        <v>0.6498687002625995</v>
+        <v>0.4485589291592267</v>
       </c>
       <c r="K79" s="2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="L79" s="2" t="n">
         <v>0</v>
@@ -4651,31 +4651,31 @@
         <v>-1</v>
       </c>
       <c r="N79" s="2" t="n">
-        <v>-0.5551685871911158</v>
+        <v>-0.8446889772863546</v>
       </c>
       <c r="O79" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, foreign_buy_3d</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
-        <v>6741</v>
+        <v>6768</v>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>91APP*-KY</t>
+          <t>志強-KY</t>
         </is>
       </c>
       <c r="C80" s="2" t="n">
         <v/>
       </c>
       <c r="D80" s="2" t="n">
-        <v>294.2601966636249</v>
+        <v>296.8022212840239</v>
       </c>
       <c r="E80" s="2" t="n">
-        <v>58</v>
+        <v>71</v>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
@@ -4686,16 +4686,16 @@
         <v>0</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>35.44733934582283</v>
+        <v>28.31496916822526</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>14.71986174869603</v>
+        <v>31.18468131202025</v>
       </c>
       <c r="J80" s="2" t="n">
-        <v>2.115214281044674</v>
+        <v>0.6498687002625995</v>
       </c>
       <c r="K80" s="2" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="L80" s="2" t="n">
         <v>0</v>
@@ -4704,31 +4704,31 @@
         <v>-1</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>-0.3032913321963202</v>
+        <v>-0.5551685871911158</v>
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, foreign_buy_3d</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
-        <v>6541</v>
+        <v>6741</v>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>泰福-KY</t>
+          <t>91APP*-KY</t>
         </is>
       </c>
       <c r="C81" s="2" t="n">
         <v/>
       </c>
       <c r="D81" s="2" t="n">
-        <v>291.4602422852631</v>
+        <v>294.2601966636249</v>
       </c>
       <c r="E81" s="2" t="n">
-        <v>40.2</v>
+        <v>58</v>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
@@ -4739,16 +4739,16 @@
         <v>0</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>48.17577178037879</v>
+        <v>35.44733934582283</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>15.23337764912538</v>
+        <v>14.71986174869603</v>
       </c>
       <c r="J81" s="2" t="n">
-        <v>0.5855210182111924</v>
+        <v>2.115214281044674</v>
       </c>
       <c r="K81" s="2" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="L81" s="2" t="n">
         <v>0</v>
@@ -4757,31 +4757,31 @@
         <v>-1</v>
       </c>
       <c r="N81" s="2" t="n">
-        <v>-0.1496840880129364</v>
+        <v>-0.3032913321963202</v>
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, kd_golden_cross, obv_uptrend</t>
+          <t>volume_break, market_above_ma60, avoid_chase, foreign_buy_3d</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
-        <v>6689</v>
+        <v>6541</v>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>伊雲谷</t>
+          <t>泰福-KY</t>
         </is>
       </c>
       <c r="C82" s="2" t="n">
         <v/>
       </c>
       <c r="D82" s="2" t="n">
-        <v>286.8016731684801</v>
+        <v>291.4602422852631</v>
       </c>
       <c r="E82" s="2" t="n">
-        <v>63.7</v>
+        <v>40.2</v>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
@@ -4792,13 +4792,13 @@
         <v>0</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>43.53195731288327</v>
+        <v>48.17577178037879</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>15.22775264435505</v>
+        <v>15.23337764912538</v>
       </c>
       <c r="J82" s="2" t="n">
-        <v>0.5414808897430692</v>
+        <v>0.5855210182111924</v>
       </c>
       <c r="K82" s="2" t="n">
         <v>0</v>
@@ -4810,7 +4810,7 @@
         <v>-1</v>
       </c>
       <c r="N82" s="2" t="n">
-        <v>0.06626286980938829</v>
+        <v>-0.1496840880129364</v>
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
@@ -4820,21 +4820,21 @@
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
-        <v>6512</v>
+        <v>6689</v>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>啟發電</t>
+          <t>伊雲谷</t>
         </is>
       </c>
       <c r="C83" s="2" t="n">
         <v/>
       </c>
       <c r="D83" s="2" t="n">
-        <v>283.7432163331612</v>
+        <v>286.8016731684801</v>
       </c>
       <c r="E83" s="2" t="n">
-        <v>0</v>
+        <v>63.7</v>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
@@ -4845,13 +4845,13 @@
         <v>0</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>34.42029817827249</v>
+        <v>43.53195731288327</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>11.32185972163585</v>
+        <v>15.22775264435505</v>
       </c>
       <c r="J83" s="2" t="n">
-        <v>0.053458029572277</v>
+        <v>0.5414808897430692</v>
       </c>
       <c r="K83" s="2" t="n">
         <v>0</v>
@@ -4863,31 +4863,31 @@
         <v>-1</v>
       </c>
       <c r="N83" s="2" t="n">
-        <v>-1.686191643164382</v>
+        <v>0.06626286980938829</v>
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, kd_golden_cross, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
-        <v>6597</v>
+        <v>6512</v>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>立誠</t>
+          <t>啟發電</t>
         </is>
       </c>
       <c r="C84" s="2" t="n">
         <v/>
       </c>
       <c r="D84" s="2" t="n">
-        <v>283.6566124750229</v>
+        <v>283.7432163331612</v>
       </c>
       <c r="E84" s="2" t="n">
-        <v>68.09999999999999</v>
+        <v>0</v>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
@@ -4898,13 +4898,13 @@
         <v>0</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>51.66413806747509</v>
+        <v>34.42029817827249</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>12.02019737170371</v>
+        <v>11.32185972163585</v>
       </c>
       <c r="J84" s="2" t="n">
-        <v>0.180112012647025</v>
+        <v>0.053458029572277</v>
       </c>
       <c r="K84" s="2" t="n">
         <v>0</v>
@@ -4916,31 +4916,31 @@
         <v>-1</v>
       </c>
       <c r="N84" s="2" t="n">
-        <v>0.4093696165401352</v>
+        <v>-1.686191643164382</v>
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, ema60_gt_ema120, market_above_ma60, avoid_chase, hist_turn_positive</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
-        <v>6807</v>
+        <v>6597</v>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>峰源-KY</t>
+          <t>立誠</t>
         </is>
       </c>
       <c r="C85" s="2" t="n">
         <v/>
       </c>
       <c r="D85" s="2" t="n">
-        <v>278.3280816754893</v>
+        <v>283.6566124750229</v>
       </c>
       <c r="E85" s="2" t="n">
-        <v>33.55</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
@@ -4951,13 +4951,13 @@
         <v>0</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>49.42508213496978</v>
+        <v>51.66413806747509</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>11.83700108631758</v>
+        <v>12.02019737170371</v>
       </c>
       <c r="J85" s="2" t="n">
-        <v>1.791620233842273</v>
+        <v>0.180112012647025</v>
       </c>
       <c r="K85" s="2" t="n">
         <v>0</v>
@@ -4969,31 +4969,31 @@
         <v>-1</v>
       </c>
       <c r="N85" s="2" t="n">
-        <v>0.0663041741582263</v>
+        <v>0.4093696165401352</v>
       </c>
       <c r="O85" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, obv_uptrend</t>
+          <t>macd_golden_cross, ema60_gt_ema120, market_above_ma60, avoid_chase, hist_turn_positive</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
-        <v>6561</v>
+        <v>6807</v>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>是方</t>
+          <t>峰源-KY</t>
         </is>
       </c>
       <c r="C86" s="2" t="n">
         <v/>
       </c>
       <c r="D86" s="2" t="n">
-        <v>277.6782024357078</v>
+        <v>278.3280816754893</v>
       </c>
       <c r="E86" s="2" t="n">
-        <v>325</v>
+        <v>33.55</v>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
@@ -5004,16 +5004,16 @@
         <v>0</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>36.83034541162738</v>
+        <v>49.42508213496978</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>23.39211892990213</v>
+        <v>11.83700108631758</v>
       </c>
       <c r="J86" s="2" t="n">
-        <v>0.3124672788414944</v>
+        <v>1.791620233842273</v>
       </c>
       <c r="K86" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L86" s="2" t="n">
         <v>0</v>
@@ -5022,31 +5022,31 @@
         <v>-1</v>
       </c>
       <c r="N86" s="2" t="n">
-        <v>-0.9302431852079104</v>
+        <v>0.0663041741582263</v>
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
+          <t>volume_break, market_above_ma60, avoid_chase, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
-        <v>6515</v>
+        <v>6561</v>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>穎崴</t>
+          <t>是方</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
         <v/>
       </c>
       <c r="D87" s="2" t="n">
-        <v>276.9147648193639</v>
+        <v>277.6782024357078</v>
       </c>
       <c r="E87" s="2" t="n">
-        <v>7255</v>
+        <v>325</v>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
@@ -5057,16 +5057,16 @@
         <v>0</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>37.91085331457374</v>
+        <v>36.83034541162738</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>17.64326801730302</v>
+        <v>23.39211892990213</v>
       </c>
       <c r="J87" s="2" t="n">
-        <v>0.4750105759352148</v>
+        <v>0.3124672788414944</v>
       </c>
       <c r="K87" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L87" s="2" t="n">
         <v>0</v>
@@ -5075,31 +5075,31 @@
         <v>-1</v>
       </c>
       <c r="N87" s="2" t="n">
-        <v>-192.2576477256265</v>
+        <v>-0.9302431852079104</v>
       </c>
       <c r="O87" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
-        <v>6671</v>
+        <v>6515</v>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>三能-KY</t>
+          <t>穎崴</t>
         </is>
       </c>
       <c r="C88" s="2" t="n">
         <v/>
       </c>
       <c r="D88" s="2" t="n">
-        <v>265.3083050109508</v>
+        <v>276.9147648193639</v>
       </c>
       <c r="E88" s="2" t="n">
-        <v>24</v>
+        <v>7255</v>
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
@@ -5110,13 +5110,13 @@
         <v>0</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>27.03429742537073</v>
+        <v>37.91085331457374</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>27.8261730476947</v>
+        <v>17.64326801730302</v>
       </c>
       <c r="J88" s="2" t="n">
-        <v>1.906659171523716</v>
+        <v>0.4750105759352148</v>
       </c>
       <c r="K88" s="2" t="n">
         <v>0</v>
@@ -5128,31 +5128,31 @@
         <v>-1</v>
       </c>
       <c r="N88" s="2" t="n">
-        <v>0.0674592962638914</v>
+        <v>-192.2576477256265</v>
       </c>
       <c r="O88" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
-        <v>6568</v>
+        <v>6671</v>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>宏觀</t>
+          <t>三能-KY</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
         <v/>
       </c>
       <c r="D89" s="2" t="n">
-        <v>263.0770231408237</v>
+        <v>265.3083050109508</v>
       </c>
       <c r="E89" s="2" t="n">
-        <v>154.5</v>
+        <v>24</v>
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
@@ -5163,13 +5163,13 @@
         <v>0</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>34.24721916139113</v>
+        <v>27.03429742537073</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>39.55588681090703</v>
+        <v>27.8261730476947</v>
       </c>
       <c r="J89" s="2" t="n">
-        <v>0.3936721971680573</v>
+        <v>1.906659171523716</v>
       </c>
       <c r="K89" s="2" t="n">
         <v>0</v>
@@ -5181,31 +5181,31 @@
         <v>-1</v>
       </c>
       <c r="N89" s="2" t="n">
-        <v>1.044861377853394</v>
+        <v>0.0674592962638914</v>
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
+          <t>volume_break, market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="n">
-        <v>6722</v>
+        <v>6568</v>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>輝創</t>
+          <t>宏觀</t>
         </is>
       </c>
       <c r="C90" s="2" t="n">
         <v/>
       </c>
       <c r="D90" s="2" t="n">
-        <v>259.1884838127905</v>
+        <v>263.0770231408237</v>
       </c>
       <c r="E90" s="2" t="n">
-        <v>34.4</v>
+        <v>154.5</v>
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
@@ -5216,13 +5216,13 @@
         <v>0</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>38.16983244354773</v>
+        <v>34.24721916139113</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>39.23582142380192</v>
+        <v>39.55588681090703</v>
       </c>
       <c r="J90" s="2" t="n">
-        <v>0.9027767271715024</v>
+        <v>0.3936721971680573</v>
       </c>
       <c r="K90" s="2" t="n">
         <v>0</v>
@@ -5234,31 +5234,31 @@
         <v>-1</v>
       </c>
       <c r="N90" s="2" t="n">
-        <v>-0.009236379256752501</v>
+        <v>1.044861377853394</v>
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="n">
-        <v>6708</v>
+        <v>6722</v>
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>天擎</t>
+          <t>輝創</t>
         </is>
       </c>
       <c r="C91" s="2" t="n">
         <v/>
       </c>
       <c r="D91" s="2" t="n">
-        <v>258.8795241698588</v>
+        <v>259.1884838127905</v>
       </c>
       <c r="E91" s="2" t="n">
-        <v>39.7</v>
+        <v>34.4</v>
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
@@ -5269,16 +5269,16 @@
         <v>0</v>
       </c>
       <c r="H91" s="2" t="n">
-        <v>48.99406632952336</v>
+        <v>38.16983244354773</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>16.92080401543225</v>
+        <v>39.23582142380192</v>
       </c>
       <c r="J91" s="2" t="n">
-        <v>1.114997778920603</v>
+        <v>0.9027767271715024</v>
       </c>
       <c r="K91" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L91" s="2" t="n">
         <v>0</v>
@@ -5287,31 +5287,31 @@
         <v>-1</v>
       </c>
       <c r="N91" s="2" t="n">
-        <v>-0.038279914852318</v>
+        <v>-0.009236379256752501</v>
       </c>
       <c r="O91" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, kd_golden_cross, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="n">
-        <v>6720</v>
+        <v>6708</v>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>久昌</t>
+          <t>天擎</t>
         </is>
       </c>
       <c r="C92" s="2" t="n">
         <v/>
       </c>
       <c r="D92" s="2" t="n">
-        <v>255.5374836617586</v>
+        <v>258.8795241698588</v>
       </c>
       <c r="E92" s="2" t="n">
-        <v>140</v>
+        <v>39.7</v>
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
@@ -5322,16 +5322,16 @@
         <v>0</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>44.63680552844105</v>
+        <v>48.99406632952336</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>20.13249140911688</v>
+        <v>16.92080401543225</v>
       </c>
       <c r="J92" s="2" t="n">
-        <v>0.5134134192445122</v>
+        <v>1.114997778920603</v>
       </c>
       <c r="K92" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L92" s="2" t="n">
         <v>0</v>
@@ -5340,31 +5340,31 @@
         <v>-1</v>
       </c>
       <c r="N92" s="2" t="n">
-        <v>0.2232482370700688</v>
+        <v>-0.038279914852318</v>
       </c>
       <c r="O92" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, kd_golden_cross, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="n">
-        <v>6821</v>
+        <v>6720</v>
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>聯寶</t>
+          <t>久昌</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
         <v/>
       </c>
       <c r="D93" s="2" t="n">
-        <v>253.8581053790432</v>
+        <v>255.5374836617586</v>
       </c>
       <c r="E93" s="2" t="n">
-        <v>48.45</v>
+        <v>140</v>
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
@@ -5375,13 +5375,13 @@
         <v>0</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>29.89075882142138</v>
+        <v>44.63680552844105</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>18.58582855737298</v>
+        <v>20.13249140911688</v>
       </c>
       <c r="J93" s="2" t="n">
-        <v>0.2214312964668881</v>
+        <v>0.5134134192445122</v>
       </c>
       <c r="K93" s="2" t="n">
         <v>0</v>
@@ -5393,31 +5393,31 @@
         <v>-1</v>
       </c>
       <c r="N93" s="2" t="n">
-        <v>-1.593919773286935</v>
+        <v>0.2232482370700688</v>
       </c>
       <c r="O93" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="n">
-        <v>6788</v>
+        <v>6821</v>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>華景電</t>
+          <t>聯寶</t>
         </is>
       </c>
       <c r="C94" s="2" t="n">
         <v/>
       </c>
       <c r="D94" s="2" t="n">
-        <v>253.6344658312614</v>
+        <v>253.8581053790432</v>
       </c>
       <c r="E94" s="2" t="n">
-        <v>391</v>
+        <v>48.45</v>
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
@@ -5428,16 +5428,16 @@
         <v>0</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>41.38643898572529</v>
+        <v>29.89075882142138</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>13.19646394389389</v>
+        <v>18.58582855737298</v>
       </c>
       <c r="J94" s="2" t="n">
-        <v>0.5120848318460797</v>
+        <v>0.2214312964668881</v>
       </c>
       <c r="K94" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L94" s="2" t="n">
         <v>0</v>
@@ -5446,7 +5446,7 @@
         <v>-1</v>
       </c>
       <c r="N94" s="2" t="n">
-        <v>-6.26247001264891</v>
+        <v>-1.593919773286935</v>
       </c>
       <c r="O94" s="2" t="inlineStr">
         <is>
@@ -5456,21 +5456,21 @@
     </row>
     <row r="95">
       <c r="A95" s="2" t="n">
-        <v>6674</v>
+        <v>6788</v>
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>鋐寶科技</t>
+          <t>華景電</t>
         </is>
       </c>
       <c r="C95" s="2" t="n">
         <v/>
       </c>
       <c r="D95" s="2" t="n">
-        <v>252.0071259665179</v>
+        <v>253.6344658312614</v>
       </c>
       <c r="E95" s="2" t="n">
-        <v>16.05</v>
+        <v>391</v>
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
@@ -5481,16 +5481,16 @@
         <v>0</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>31.07236596301401</v>
+        <v>41.38643898572529</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>21.35817874158171</v>
+        <v>13.19646394389389</v>
       </c>
       <c r="J95" s="2" t="n">
-        <v>2.254231052244297</v>
+        <v>0.5120848318460797</v>
       </c>
       <c r="K95" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L95" s="2" t="n">
         <v>0</v>
@@ -5499,31 +5499,31 @@
         <v>-1</v>
       </c>
       <c r="N95" s="2" t="n">
-        <v>-0.0814265374288865</v>
+        <v>-6.26247001264891</v>
       </c>
       <c r="O95" s="2" t="inlineStr">
         <is>
-          <t>volume_break, market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="n">
-        <v>6550</v>
+        <v>6674</v>
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>北極星藥業-KY</t>
+          <t>鋐寶科技</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
         <v/>
       </c>
       <c r="D96" s="2" t="n">
-        <v>249.8057436248971</v>
+        <v>252.0071259665179</v>
       </c>
       <c r="E96" s="2" t="n">
-        <v>12.5</v>
+        <v>16.05</v>
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
@@ -5534,13 +5534,13 @@
         <v>0</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>38.52809340817095</v>
+        <v>31.07236596301401</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>20.75496293497697</v>
+        <v>21.35817874158171</v>
       </c>
       <c r="J96" s="2" t="n">
-        <v>0.5842216948447265</v>
+        <v>2.254231052244297</v>
       </c>
       <c r="K96" s="2" t="n">
         <v>0</v>
@@ -5552,31 +5552,31 @@
         <v>-1</v>
       </c>
       <c r="N96" s="2" t="n">
-        <v>0.0062831642802622</v>
+        <v>-0.0814265374288865</v>
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
+          <t>volume_break, market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="n">
-        <v>6498</v>
+        <v>6550</v>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>久禾光</t>
+          <t>北極星藥業-KY</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
         <v/>
       </c>
       <c r="D97" s="2" t="n">
-        <v>244.8801149338972</v>
+        <v>249.8057436248971</v>
       </c>
       <c r="E97" s="2" t="n">
-        <v>85.5</v>
+        <v>12.5</v>
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
@@ -5587,13 +5587,13 @@
         <v>0</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>33.83237328252054</v>
+        <v>38.52809340817095</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>21.31568695566191</v>
+        <v>20.75496293497697</v>
       </c>
       <c r="J97" s="2" t="n">
-        <v>0.3372138439608252</v>
+        <v>0.5842216948447265</v>
       </c>
       <c r="K97" s="2" t="n">
         <v>0</v>
@@ -5605,31 +5605,31 @@
         <v>-1</v>
       </c>
       <c r="N97" s="2" t="n">
-        <v>-1.000830795936182</v>
+        <v>0.0062831642802622</v>
       </c>
       <c r="O97" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="n">
-        <v>6560</v>
+        <v>6498</v>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>欣普羅</t>
+          <t>久禾光</t>
         </is>
       </c>
       <c r="C98" s="2" t="n">
         <v/>
       </c>
       <c r="D98" s="2" t="n">
-        <v>240.9983357698996</v>
+        <v>244.8801149338972</v>
       </c>
       <c r="E98" s="2" t="n">
-        <v>35.55</v>
+        <v>85.5</v>
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
@@ -5640,16 +5640,16 @@
         <v>0</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>34.79805276120388</v>
+        <v>33.83237328252054</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>23.34472686673146</v>
+        <v>21.31568695566191</v>
       </c>
       <c r="J98" s="2" t="n">
-        <v>0.5691621469732571</v>
+        <v>0.3372138439608252</v>
       </c>
       <c r="K98" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L98" s="2" t="n">
         <v>0</v>
@@ -5658,31 +5658,31 @@
         <v>-1</v>
       </c>
       <c r="N98" s="2" t="n">
-        <v>-0.4093625724875958</v>
+        <v>-1.000830795936182</v>
       </c>
       <c r="O98" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="n">
-        <v>6838</v>
+        <v>6560</v>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>台新藥</t>
+          <t>欣普羅</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
         <v/>
       </c>
       <c r="D99" s="2" t="n">
-        <v>239.1001293203865</v>
+        <v>240.9983357698996</v>
       </c>
       <c r="E99" s="2" t="n">
-        <v>24.2</v>
+        <v>35.55</v>
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
@@ -5693,16 +5693,16 @@
         <v>0</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>46.0305190333092</v>
+        <v>34.79805276120388</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>11.29061050627273</v>
+        <v>23.34472686673146</v>
       </c>
       <c r="J99" s="2" t="n">
-        <v>0.5232827107120422</v>
+        <v>0.5691621469732571</v>
       </c>
       <c r="K99" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L99" s="2" t="n">
         <v>0</v>
@@ -5711,31 +5711,31 @@
         <v>-1</v>
       </c>
       <c r="N99" s="2" t="n">
-        <v>0.0540316209743964</v>
+        <v>-0.4093625724875958</v>
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, kd_golden_cross, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="n">
-        <v>6592</v>
+        <v>6838</v>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>和潤企業</t>
+          <t>台新藥</t>
         </is>
       </c>
       <c r="C100" s="2" t="n">
         <v/>
       </c>
       <c r="D100" s="2" t="n">
-        <v>237.937332471623</v>
+        <v>239.1001293203865</v>
       </c>
       <c r="E100" s="2" t="n">
-        <v>60.4</v>
+        <v>24.2</v>
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
@@ -5746,13 +5746,13 @@
         <v>0</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>43.07027713832887</v>
+        <v>46.0305190333092</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>24.69857441325158</v>
+        <v>11.29061050627273</v>
       </c>
       <c r="J100" s="2" t="n">
-        <v>1.461845164225781</v>
+        <v>0.5232827107120422</v>
       </c>
       <c r="K100" s="2" t="n">
         <v>0</v>
@@ -5764,31 +5764,31 @@
         <v>-1</v>
       </c>
       <c r="N100" s="2" t="n">
-        <v>-0.3050627205985258</v>
+        <v>0.0540316209743964</v>
       </c>
       <c r="O100" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, kd_golden_cross, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="n">
-        <v>6803</v>
+        <v>6592</v>
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>崑鼎</t>
+          <t>和潤企業</t>
         </is>
       </c>
       <c r="C101" s="2" t="n">
         <v/>
       </c>
       <c r="D101" s="2" t="n">
-        <v>235.3575815954785</v>
+        <v>237.937332471623</v>
       </c>
       <c r="E101" s="2" t="n">
-        <v>270.5</v>
+        <v>60.4</v>
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
@@ -5799,13 +5799,13 @@
         <v>0</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>24.65015709199119</v>
+        <v>43.07027713832887</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>42.12690928664343</v>
+        <v>24.69857441325158</v>
       </c>
       <c r="J101" s="2" t="n">
-        <v>0.3502267484669848</v>
+        <v>1.461845164225781</v>
       </c>
       <c r="K101" s="2" t="n">
         <v>0</v>
@@ -5817,31 +5817,31 @@
         <v>-1</v>
       </c>
       <c r="N101" s="2" t="n">
-        <v>-1.625282801350652</v>
+        <v>-0.3050627205985258</v>
       </c>
       <c r="O101" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="n">
-        <v>6794</v>
+        <v>6803</v>
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>向榮生技-創</t>
+          <t>崑鼎</t>
         </is>
       </c>
       <c r="C102" s="2" t="n">
         <v/>
       </c>
       <c r="D102" s="2" t="n">
-        <v>234.5974983014461</v>
+        <v>235.3575815954785</v>
       </c>
       <c r="E102" s="2" t="n">
-        <v>79.09999999999999</v>
+        <v>270.5</v>
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
@@ -5852,13 +5852,13 @@
         <v>0</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>46.29197659546669</v>
+        <v>24.65015709199119</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>17.12534270737977</v>
+        <v>42.12690928664343</v>
       </c>
       <c r="J102" s="2" t="n">
-        <v>0.9022569958505136</v>
+        <v>0.3502267484669848</v>
       </c>
       <c r="K102" s="2" t="n">
         <v>0</v>
@@ -5870,31 +5870,31 @@
         <v>-1</v>
       </c>
       <c r="N102" s="2" t="n">
-        <v>-0.0530345965821242</v>
+        <v>-1.625282801350652</v>
       </c>
       <c r="O102" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="n">
-        <v>6761</v>
+        <v>6794</v>
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>穩得</t>
+          <t>向榮生技-創</t>
         </is>
       </c>
       <c r="C103" s="2" t="n">
         <v/>
       </c>
       <c r="D103" s="2" t="n">
-        <v>232.5603724330552</v>
+        <v>234.5974983014461</v>
       </c>
       <c r="E103" s="2" t="n">
-        <v>171.5</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
@@ -5905,13 +5905,13 @@
         <v>0</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>39.05722984644048</v>
+        <v>46.29197659546669</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>14.26193669277529</v>
+        <v>17.12534270737977</v>
       </c>
       <c r="J103" s="2" t="n">
-        <v>0.4774663734979514</v>
+        <v>0.9022569958505136</v>
       </c>
       <c r="K103" s="2" t="n">
         <v>0</v>
@@ -5923,31 +5923,31 @@
         <v>-1</v>
       </c>
       <c r="N103" s="2" t="n">
-        <v>-2.2985697613505</v>
+        <v>-0.0530345965821242</v>
       </c>
       <c r="O103" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="n">
-        <v>6625</v>
+        <v>6761</v>
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>必應</t>
+          <t>穩得</t>
         </is>
       </c>
       <c r="C104" s="2" t="n">
         <v/>
       </c>
       <c r="D104" s="2" t="n">
-        <v>231.9383994193332</v>
+        <v>232.5603724330552</v>
       </c>
       <c r="E104" s="2" t="n">
-        <v>78.3</v>
+        <v>171.5</v>
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
@@ -5958,13 +5958,13 @@
         <v>0</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>52.55896606243697</v>
+        <v>39.05722984644048</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>22.68908525536767</v>
+        <v>14.26193669277529</v>
       </c>
       <c r="J104" s="2" t="n">
-        <v>0.476362320555696</v>
+        <v>0.4774663734979514</v>
       </c>
       <c r="K104" s="2" t="n">
         <v>0</v>
@@ -5976,31 +5976,31 @@
         <v>-1</v>
       </c>
       <c r="N104" s="2" t="n">
-        <v>-0.1936123444092289</v>
+        <v>-2.2985697613505</v>
       </c>
       <c r="O104" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending, above_ichimoku_cloud</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="n">
-        <v>6776</v>
+        <v>6625</v>
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>展碁國際</t>
+          <t>必應</t>
         </is>
       </c>
       <c r="C105" s="2" t="n">
         <v/>
       </c>
       <c r="D105" s="2" t="n">
-        <v>228.8302949368482</v>
+        <v>231.9383994193332</v>
       </c>
       <c r="E105" s="2" t="n">
-        <v>55.4</v>
+        <v>78.3</v>
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
@@ -6011,13 +6011,13 @@
         <v>0</v>
       </c>
       <c r="H105" s="2" t="n">
-        <v>44.86287803481545</v>
+        <v>52.55896606243697</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>14.79185965641763</v>
+        <v>22.68908525536767</v>
       </c>
       <c r="J105" s="2" t="n">
-        <v>0.4513310011390415</v>
+        <v>0.476362320555696</v>
       </c>
       <c r="K105" s="2" t="n">
         <v>0</v>
@@ -6029,31 +6029,31 @@
         <v>-1</v>
       </c>
       <c r="N105" s="2" t="n">
-        <v>0.0801635202756705</v>
+        <v>-0.1936123444092289</v>
       </c>
       <c r="O105" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, adx_trending, above_ichimoku_cloud</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="n">
-        <v>6715</v>
+        <v>6776</v>
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>嘉基</t>
+          <t>展碁國際</t>
         </is>
       </c>
       <c r="C106" s="2" t="n">
         <v/>
       </c>
       <c r="D106" s="2" t="n">
-        <v>220.7445224238494</v>
+        <v>228.8302949368482</v>
       </c>
       <c r="E106" s="2" t="n">
-        <v>374</v>
+        <v>55.4</v>
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
@@ -6064,13 +6064,13 @@
         <v>0</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>39.43945440686664</v>
+        <v>44.86287803481545</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>15.85054159028268</v>
+        <v>14.79185965641763</v>
       </c>
       <c r="J106" s="2" t="n">
-        <v>0.4235315708375018</v>
+        <v>0.4513310011390415</v>
       </c>
       <c r="K106" s="2" t="n">
         <v>0</v>
@@ -6082,31 +6082,31 @@
         <v>-1</v>
       </c>
       <c r="N106" s="2" t="n">
-        <v>-11.82046835780611</v>
+        <v>0.0801635202756705</v>
       </c>
       <c r="O106" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="n">
-        <v>6754</v>
+        <v>6715</v>
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>匯僑設計</t>
+          <t>嘉基</t>
         </is>
       </c>
       <c r="C107" s="2" t="n">
         <v/>
       </c>
       <c r="D107" s="2" t="n">
-        <v>218.9659081876185</v>
+        <v>220.7445224238494</v>
       </c>
       <c r="E107" s="2" t="n">
-        <v>43.55</v>
+        <v>374</v>
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
@@ -6117,13 +6117,13 @@
         <v>0</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>47.89794226641228</v>
+        <v>39.43945440686664</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>17.35551806250441</v>
+        <v>15.85054159028268</v>
       </c>
       <c r="J107" s="2" t="n">
-        <v>0.8661863795444307</v>
+        <v>0.4235315708375018</v>
       </c>
       <c r="K107" s="2" t="n">
         <v>0</v>
@@ -6135,31 +6135,31 @@
         <v>-1</v>
       </c>
       <c r="N107" s="2" t="n">
-        <v>-0.2129337114443878</v>
+        <v>-11.82046835780611</v>
       </c>
       <c r="O107" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="n">
-        <v>6706</v>
+        <v>6754</v>
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>惠特</t>
+          <t>匯僑設計</t>
         </is>
       </c>
       <c r="C108" s="2" t="n">
         <v/>
       </c>
       <c r="D108" s="2" t="n">
-        <v>218.8322945014885</v>
+        <v>218.9659081876185</v>
       </c>
       <c r="E108" s="2" t="n">
-        <v>128.5</v>
+        <v>43.55</v>
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
@@ -6170,13 +6170,13 @@
         <v>0</v>
       </c>
       <c r="H108" s="2" t="n">
-        <v>33.9617500281434</v>
+        <v>47.89794226641228</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>19.82992277580565</v>
+        <v>17.35551806250441</v>
       </c>
       <c r="J108" s="2" t="n">
-        <v>0.4518652610181384</v>
+        <v>0.8661863795444307</v>
       </c>
       <c r="K108" s="2" t="n">
         <v>0</v>
@@ -6188,31 +6188,31 @@
         <v>-1</v>
       </c>
       <c r="N108" s="2" t="n">
-        <v>-2.063481822853021</v>
+        <v>-0.2129337114443878</v>
       </c>
       <c r="O108" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="n">
-        <v>6698</v>
+        <v>6706</v>
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>旭暉應材</t>
+          <t>惠特</t>
         </is>
       </c>
       <c r="C109" s="2" t="n">
         <v/>
       </c>
       <c r="D109" s="2" t="n">
-        <v>215.2171225938938</v>
+        <v>218.8322945014885</v>
       </c>
       <c r="E109" s="2" t="n">
-        <v>39.15</v>
+        <v>128.5</v>
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
@@ -6223,13 +6223,13 @@
         <v>0</v>
       </c>
       <c r="H109" s="2" t="n">
-        <v>45.8232580642138</v>
+        <v>33.9617500281434</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>24.07675205038112</v>
+        <v>19.82992277580565</v>
       </c>
       <c r="J109" s="2" t="n">
-        <v>0.1998143501544385</v>
+        <v>0.4518652610181384</v>
       </c>
       <c r="K109" s="2" t="n">
         <v>0</v>
@@ -6241,31 +6241,31 @@
         <v>-1</v>
       </c>
       <c r="N109" s="2" t="n">
-        <v>-0.7397244149827634</v>
+        <v>-2.063481822853021</v>
       </c>
       <c r="O109" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="n">
-        <v>6792</v>
+        <v>6698</v>
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>詠業</t>
+          <t>旭暉應材</t>
         </is>
       </c>
       <c r="C110" s="2" t="n">
         <v/>
       </c>
       <c r="D110" s="2" t="n">
-        <v>212.4838843783731</v>
+        <v>215.2171225938938</v>
       </c>
       <c r="E110" s="2" t="n">
-        <v>58.2</v>
+        <v>39.15</v>
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
@@ -6276,13 +6276,13 @@
         <v>0</v>
       </c>
       <c r="H110" s="2" t="n">
-        <v>36.39474571464705</v>
+        <v>45.8232580642138</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>18.38277520156264</v>
+        <v>24.07675205038112</v>
       </c>
       <c r="J110" s="2" t="n">
-        <v>0.5155635754333956</v>
+        <v>0.1998143501544385</v>
       </c>
       <c r="K110" s="2" t="n">
         <v>0</v>
@@ -6294,31 +6294,31 @@
         <v>-1</v>
       </c>
       <c r="N110" s="2" t="n">
-        <v>-0.8855725425486696</v>
+        <v>-0.7397244149827634</v>
       </c>
       <c r="O110" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="n">
-        <v>6667</v>
+        <v>6792</v>
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>信紘科</t>
+          <t>詠業</t>
         </is>
       </c>
       <c r="C111" s="2" t="n">
         <v/>
       </c>
       <c r="D111" s="2" t="n">
-        <v>211.7287864315561</v>
+        <v>212.4838843783731</v>
       </c>
       <c r="E111" s="2" t="n">
-        <v>258.5</v>
+        <v>58.2</v>
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
@@ -6329,16 +6329,16 @@
         <v>0</v>
       </c>
       <c r="H111" s="2" t="n">
-        <v>44.966096985913</v>
+        <v>36.39474571464705</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>12.6852093332146</v>
+        <v>18.38277520156264</v>
       </c>
       <c r="J111" s="2" t="n">
-        <v>0.3820644592901437</v>
+        <v>0.5155635754333956</v>
       </c>
       <c r="K111" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L111" s="2" t="n">
         <v>0</v>
@@ -6347,31 +6347,31 @@
         <v>-1</v>
       </c>
       <c r="N111" s="2" t="n">
-        <v>-1.729225787859067</v>
+        <v>-0.8855725425486696</v>
       </c>
       <c r="O111" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="n">
-        <v>6581</v>
+        <v>6667</v>
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>鋼聯</t>
+          <t>信紘科</t>
         </is>
       </c>
       <c r="C112" s="2" t="n">
         <v/>
       </c>
       <c r="D112" s="2" t="n">
-        <v>209.0004093267832</v>
+        <v>211.7287864315561</v>
       </c>
       <c r="E112" s="2" t="n">
-        <v>108</v>
+        <v>258.5</v>
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
@@ -6382,16 +6382,16 @@
         <v>0</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>52.57611758899868</v>
+        <v>44.966096985913</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>10.08401216618641</v>
+        <v>12.6852093332146</v>
       </c>
       <c r="J112" s="2" t="n">
-        <v>1.1552249741597</v>
+        <v>0.3820644592901437</v>
       </c>
       <c r="K112" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L112" s="2" t="n">
         <v>0</v>
@@ -6400,31 +6400,31 @@
         <v>-1</v>
       </c>
       <c r="N112" s="2" t="n">
-        <v>0.1674529354585579</v>
+        <v>-1.729225787859067</v>
       </c>
       <c r="O112" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="n">
-        <v>6531</v>
+        <v>6581</v>
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>愛普*</t>
+          <t>鋼聯</t>
         </is>
       </c>
       <c r="C113" s="2" t="n">
         <v/>
       </c>
       <c r="D113" s="2" t="n">
-        <v>208.6341960813816</v>
+        <v>209.0004093267832</v>
       </c>
       <c r="E113" s="2" t="n">
-        <v>943</v>
+        <v>108</v>
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
@@ -6435,13 +6435,13 @@
         <v>0</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>48.6504212344406</v>
+        <v>52.57611758899868</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>17.044964490526</v>
+        <v>10.08401216618641</v>
       </c>
       <c r="J113" s="2" t="n">
-        <v>0.4944684600542852</v>
+        <v>1.1552249741597</v>
       </c>
       <c r="K113" s="2" t="n">
         <v>0</v>
@@ -6453,31 +6453,31 @@
         <v>-1</v>
       </c>
       <c r="N113" s="2" t="n">
-        <v>-11.27975853628699</v>
+        <v>0.1674529354585579</v>
       </c>
       <c r="O113" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="n">
-        <v>6591</v>
+        <v>6531</v>
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>動力-KY</t>
+          <t>愛普*</t>
         </is>
       </c>
       <c r="C114" s="2" t="n">
         <v/>
       </c>
       <c r="D114" s="2" t="n">
-        <v>203.7080826389992</v>
+        <v>208.6341960813816</v>
       </c>
       <c r="E114" s="2" t="n">
-        <v>45.35</v>
+        <v>943</v>
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
@@ -6488,13 +6488,13 @@
         <v>0</v>
       </c>
       <c r="H114" s="2" t="n">
-        <v>23.7504771000064</v>
+        <v>48.6504212344406</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>29.7537529015491</v>
+        <v>17.044964490526</v>
       </c>
       <c r="J114" s="2" t="n">
-        <v>0.6836793160502818</v>
+        <v>0.4944684600542852</v>
       </c>
       <c r="K114" s="2" t="n">
         <v>0</v>
@@ -6506,31 +6506,31 @@
         <v>-1</v>
       </c>
       <c r="N114" s="2" t="n">
-        <v>-0.9153935160763756</v>
+        <v>-11.27975853628699</v>
       </c>
       <c r="O114" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="n">
-        <v>6796</v>
+        <v>6591</v>
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
-          <t>晉弘</t>
+          <t>動力-KY</t>
         </is>
       </c>
       <c r="C115" s="2" t="n">
         <v/>
       </c>
       <c r="D115" s="2" t="n">
-        <v>199.224071196507</v>
+        <v>203.7080826389992</v>
       </c>
       <c r="E115" s="2" t="n">
-        <v>59.7</v>
+        <v>45.35</v>
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
@@ -6541,13 +6541,13 @@
         <v>0</v>
       </c>
       <c r="H115" s="2" t="n">
-        <v>51.30861516790864</v>
+        <v>23.7504771000064</v>
       </c>
       <c r="I115" s="2" t="n">
-        <v>19.75965359173369</v>
+        <v>29.7537529015491</v>
       </c>
       <c r="J115" s="2" t="n">
-        <v>0.8970248398234659</v>
+        <v>0.6836793160502818</v>
       </c>
       <c r="K115" s="2" t="n">
         <v>0</v>
@@ -6559,31 +6559,31 @@
         <v>-1</v>
       </c>
       <c r="N115" s="2" t="n">
-        <v>0.3656424941579228</v>
+        <v>-0.9153935160763756</v>
       </c>
       <c r="O115" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="n">
-        <v>6695</v>
+        <v>6796</v>
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>芯鼎</t>
+          <t>晉弘</t>
         </is>
       </c>
       <c r="C116" s="2" t="n">
         <v/>
       </c>
       <c r="D116" s="2" t="n">
-        <v>185.1291710776382</v>
+        <v>199.224071196507</v>
       </c>
       <c r="E116" s="2" t="n">
-        <v>57.6</v>
+        <v>59.7</v>
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
@@ -6594,13 +6594,13 @@
         <v>0</v>
       </c>
       <c r="H116" s="2" t="n">
-        <v>52.27485283537935</v>
+        <v>51.30861516790864</v>
       </c>
       <c r="I116" s="2" t="n">
-        <v>17.90594338417606</v>
+        <v>19.75965359173369</v>
       </c>
       <c r="J116" s="2" t="n">
-        <v>0.7301857003083591</v>
+        <v>0.8970248398234659</v>
       </c>
       <c r="K116" s="2" t="n">
         <v>0</v>
@@ -6612,31 +6612,31 @@
         <v>-1</v>
       </c>
       <c r="N116" s="2" t="n">
-        <v>-0.7834720168422193</v>
+        <v>0.3656424941579228</v>
       </c>
       <c r="O116" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="n">
-        <v>6605</v>
+        <v>6695</v>
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t>帝寶</t>
+          <t>芯鼎</t>
         </is>
       </c>
       <c r="C117" s="2" t="n">
         <v/>
       </c>
       <c r="D117" s="2" t="n">
-        <v>179.8434156287256</v>
+        <v>185.1291710776382</v>
       </c>
       <c r="E117" s="2" t="n">
-        <v>128.5</v>
+        <v>57.6</v>
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
@@ -6647,13 +6647,13 @@
         <v>0</v>
       </c>
       <c r="H117" s="2" t="n">
-        <v>38.39062838849312</v>
+        <v>52.27485283537935</v>
       </c>
       <c r="I117" s="2" t="n">
-        <v>17.08908006432618</v>
+        <v>17.90594338417606</v>
       </c>
       <c r="J117" s="2" t="n">
-        <v>0.3689546474986174</v>
+        <v>0.7301857003083591</v>
       </c>
       <c r="K117" s="2" t="n">
         <v>0</v>
@@ -6665,31 +6665,31 @@
         <v>-1</v>
       </c>
       <c r="N117" s="2" t="n">
-        <v>-1.26392190456033</v>
+        <v>-0.7834720168422193</v>
       </c>
       <c r="O117" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="n">
-        <v>6770</v>
+        <v>6605</v>
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>力積電</t>
+          <t>帝寶</t>
         </is>
       </c>
       <c r="C118" s="2" t="n">
         <v/>
       </c>
       <c r="D118" s="2" t="n">
-        <v>176.7746543033423</v>
+        <v>179.8434156287256</v>
       </c>
       <c r="E118" s="2" t="n">
-        <v>76.09999999999999</v>
+        <v>128.5</v>
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
@@ -6700,13 +6700,13 @@
         <v>0</v>
       </c>
       <c r="H118" s="2" t="n">
-        <v>54.22017466469468</v>
+        <v>38.39062838849312</v>
       </c>
       <c r="I118" s="2" t="n">
-        <v>15.04535307933507</v>
+        <v>17.08908006432618</v>
       </c>
       <c r="J118" s="2" t="n">
-        <v>0.8421519597477961</v>
+        <v>0.3689546474986174</v>
       </c>
       <c r="K118" s="2" t="n">
         <v>0</v>
@@ -6718,31 +6718,31 @@
         <v>-1</v>
       </c>
       <c r="N118" s="2" t="n">
-        <v>-0.7812642293747033</v>
+        <v>-1.26392190456033</v>
       </c>
       <c r="O118" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="n">
-        <v>6546</v>
+        <v>6770</v>
       </c>
       <c r="B119" s="2" t="inlineStr">
         <is>
-          <t>正基</t>
+          <t>力積電</t>
         </is>
       </c>
       <c r="C119" s="2" t="n">
         <v/>
       </c>
       <c r="D119" s="2" t="n">
-        <v>163.3302334954933</v>
+        <v>176.7746543033423</v>
       </c>
       <c r="E119" s="2" t="n">
-        <v>65.5</v>
+        <v>76.09999999999999</v>
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
@@ -6753,16 +6753,16 @@
         <v>0</v>
       </c>
       <c r="H119" s="2" t="n">
-        <v>38.62970640733516</v>
+        <v>54.22017466469468</v>
       </c>
       <c r="I119" s="2" t="n">
-        <v>15.80627851805784</v>
+        <v>15.04535307933507</v>
       </c>
       <c r="J119" s="2" t="n">
-        <v>0.3483807078441215</v>
+        <v>0.8421519597477961</v>
       </c>
       <c r="K119" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L119" s="2" t="n">
         <v>0</v>
@@ -6771,31 +6771,31 @@
         <v>-1</v>
       </c>
       <c r="N119" s="2" t="n">
-        <v>-0.5621963515127277</v>
+        <v>-0.7812642293747033</v>
       </c>
       <c r="O119" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>ema60_gt_ema120, market_above_ma60, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="n">
-        <v>6558</v>
+        <v>6546</v>
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>興能高</t>
+          <t>正基</t>
         </is>
       </c>
       <c r="C120" s="2" t="n">
         <v/>
       </c>
       <c r="D120" s="2" t="n">
-        <v>140.4896760201823</v>
+        <v>163.3302334954933</v>
       </c>
       <c r="E120" s="2" t="n">
-        <v>29.15</v>
+        <v>65.5</v>
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
@@ -6806,16 +6806,16 @@
         <v>0</v>
       </c>
       <c r="H120" s="2" t="n">
-        <v>43.7783058907513</v>
+        <v>38.62970640733516</v>
       </c>
       <c r="I120" s="2" t="n">
-        <v>15.02390955445812</v>
+        <v>15.80627851805784</v>
       </c>
       <c r="J120" s="2" t="n">
-        <v>0.3055180328500801</v>
+        <v>0.3483807078441215</v>
       </c>
       <c r="K120" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L120" s="2" t="n">
         <v>0</v>
@@ -6824,31 +6824,31 @@
         <v>-1</v>
       </c>
       <c r="N120" s="2" t="n">
-        <v>-0.0124812082186298</v>
+        <v>-0.5621963515127277</v>
       </c>
       <c r="O120" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="n">
-        <v>6771</v>
+        <v>6558</v>
       </c>
       <c r="B121" s="2" t="inlineStr">
         <is>
-          <t>平和環保-創</t>
+          <t>興能高</t>
         </is>
       </c>
       <c r="C121" s="2" t="n">
         <v/>
       </c>
       <c r="D121" s="2" t="n">
-        <v>137.5268862935678</v>
+        <v>140.4896760201823</v>
       </c>
       <c r="E121" s="2" t="n">
-        <v>39.3</v>
+        <v>29.15</v>
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
@@ -6859,13 +6859,13 @@
         <v>0</v>
       </c>
       <c r="H121" s="2" t="n">
-        <v>42.08809428764791</v>
+        <v>43.7783058907513</v>
       </c>
       <c r="I121" s="2" t="n">
-        <v>17.78060647098754</v>
+        <v>15.02390955445812</v>
       </c>
       <c r="J121" s="2" t="n">
-        <v>0.1159963287161961</v>
+        <v>0.3055180328500801</v>
       </c>
       <c r="K121" s="2" t="n">
         <v>0</v>
@@ -6877,31 +6877,31 @@
         <v>-1</v>
       </c>
       <c r="N121" s="2" t="n">
-        <v>0.0514804729917596</v>
+        <v>-0.0124812082186298</v>
       </c>
       <c r="O121" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
+          <t>market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="n">
-        <v>6657</v>
+        <v>6771</v>
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>華安</t>
+          <t>平和環保-創</t>
         </is>
       </c>
       <c r="C122" s="2" t="n">
         <v/>
       </c>
       <c r="D122" s="2" t="n">
-        <v>135.9159622283808</v>
+        <v>137.5268862935678</v>
       </c>
       <c r="E122" s="2" t="n">
-        <v>35</v>
+        <v>39.3</v>
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
@@ -6912,13 +6912,13 @@
         <v>0</v>
       </c>
       <c r="H122" s="2" t="n">
-        <v>44.32564922198883</v>
+        <v>42.08809428764791</v>
       </c>
       <c r="I122" s="2" t="n">
-        <v>18.97659443665826</v>
+        <v>17.78060647098754</v>
       </c>
       <c r="J122" s="2" t="n">
-        <v>0.655121939058369</v>
+        <v>0.1159963287161961</v>
       </c>
       <c r="K122" s="2" t="n">
         <v>0</v>
@@ -6930,31 +6930,31 @@
         <v>-1</v>
       </c>
       <c r="N122" s="2" t="n">
-        <v>-0.0262164573998457</v>
+        <v>0.0514804729917596</v>
       </c>
       <c r="O122" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, mfi_strong</t>
+          <t>market_above_ma60, avoid_chase, kd_golden_cross</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="n">
-        <v>6552</v>
+        <v>6657</v>
       </c>
       <c r="B123" s="2" t="inlineStr">
         <is>
-          <t>易華電</t>
+          <t>華安</t>
         </is>
       </c>
       <c r="C123" s="2" t="n">
         <v/>
       </c>
       <c r="D123" s="2" t="n">
-        <v>134.5997514065583</v>
+        <v>135.9159622283808</v>
       </c>
       <c r="E123" s="2" t="n">
-        <v>28.2</v>
+        <v>35</v>
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
@@ -6965,13 +6965,13 @@
         <v>0</v>
       </c>
       <c r="H123" s="2" t="n">
-        <v>41.82653752192287</v>
+        <v>44.32564922198883</v>
       </c>
       <c r="I123" s="2" t="n">
-        <v>13.11522793123545</v>
+        <v>18.97659443665826</v>
       </c>
       <c r="J123" s="2" t="n">
-        <v>0.5575372223251798</v>
+        <v>0.655121939058369</v>
       </c>
       <c r="K123" s="2" t="n">
         <v>0</v>
@@ -6983,31 +6983,31 @@
         <v>-1</v>
       </c>
       <c r="N123" s="2" t="n">
-        <v>-0.2593394207480055</v>
+        <v>-0.0262164573998457</v>
       </c>
       <c r="O123" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, mfi_strong</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="n">
-        <v>6763</v>
+        <v>6552</v>
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t>綠界科技</t>
+          <t>易華電</t>
         </is>
       </c>
       <c r="C124" s="2" t="n">
         <v/>
       </c>
       <c r="D124" s="2" t="n">
-        <v>122.3225730553719</v>
+        <v>134.5997514065583</v>
       </c>
       <c r="E124" s="2" t="n">
-        <v>43.7</v>
+        <v>28.2</v>
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
@@ -7018,16 +7018,16 @@
         <v>0</v>
       </c>
       <c r="H124" s="2" t="n">
-        <v>37.22376145810392</v>
+        <v>41.82653752192287</v>
       </c>
       <c r="I124" s="2" t="n">
-        <v>17.75075099676165</v>
+        <v>13.11522793123545</v>
       </c>
       <c r="J124" s="2" t="n">
-        <v>0.3331254168878176</v>
+        <v>0.5575372223251798</v>
       </c>
       <c r="K124" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L124" s="2" t="n">
         <v>0</v>
@@ -7036,31 +7036,31 @@
         <v>-1</v>
       </c>
       <c r="N124" s="2" t="n">
-        <v>-0.4347044686968042</v>
+        <v>-0.2593394207480055</v>
       </c>
       <c r="O124" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="n">
-        <v>6614</v>
+        <v>6763</v>
       </c>
       <c r="B125" s="2" t="inlineStr">
         <is>
-          <t>資拓宏宇</t>
+          <t>綠界科技</t>
         </is>
       </c>
       <c r="C125" s="2" t="n">
         <v/>
       </c>
       <c r="D125" s="2" t="n">
-        <v>103.5522793126277</v>
+        <v>122.3225730553719</v>
       </c>
       <c r="E125" s="2" t="n">
-        <v>39.25</v>
+        <v>43.7</v>
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
@@ -7071,16 +7071,16 @@
         <v>0</v>
       </c>
       <c r="H125" s="2" t="n">
-        <v>41.61583660794673</v>
+        <v>37.22376145810392</v>
       </c>
       <c r="I125" s="2" t="n">
-        <v>19.78643800729449</v>
+        <v>17.75075099676165</v>
       </c>
       <c r="J125" s="2" t="n">
-        <v>1.133341928359333</v>
+        <v>0.3331254168878176</v>
       </c>
       <c r="K125" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L125" s="2" t="n">
         <v>0</v>
@@ -7089,7 +7089,7 @@
         <v>-1</v>
       </c>
       <c r="N125" s="2" t="n">
-        <v>-0.0365753553602106</v>
+        <v>-0.4347044686968042</v>
       </c>
       <c r="O125" s="2" t="inlineStr">
         <is>
@@ -7099,21 +7099,21 @@
     </row>
     <row r="126">
       <c r="A126" s="2" t="n">
-        <v>6692</v>
+        <v>6614</v>
       </c>
       <c r="B126" s="2" t="inlineStr">
         <is>
-          <t>進能服</t>
+          <t>資拓宏宇</t>
         </is>
       </c>
       <c r="C126" s="2" t="n">
         <v/>
       </c>
       <c r="D126" s="2" t="n">
-        <v>90.61611310658471</v>
+        <v>103.5522793126277</v>
       </c>
       <c r="E126" s="2" t="n">
-        <v>24.8</v>
+        <v>39.25</v>
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
@@ -7124,13 +7124,13 @@
         <v>0</v>
       </c>
       <c r="H126" s="2" t="n">
-        <v>42.15010975706134</v>
+        <v>41.61583660794673</v>
       </c>
       <c r="I126" s="2" t="n">
-        <v>12.37993747398537</v>
+        <v>19.78643800729449</v>
       </c>
       <c r="J126" s="2" t="n">
-        <v>0.2863272076772039</v>
+        <v>1.133341928359333</v>
       </c>
       <c r="K126" s="2" t="n">
         <v>0</v>
@@ -7142,7 +7142,7 @@
         <v>-1</v>
       </c>
       <c r="N126" s="2" t="n">
-        <v>-0.0250700897444002</v>
+        <v>-0.0365753553602106</v>
       </c>
       <c r="O126" s="2" t="inlineStr">
         <is>
@@ -7152,52 +7152,105 @@
     </row>
     <row r="127">
       <c r="A127" s="2" t="n">
+        <v>6692</v>
+      </c>
+      <c r="B127" s="2" t="inlineStr">
+        <is>
+          <t>進能服</t>
+        </is>
+      </c>
+      <c r="C127" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D127" s="2" t="n">
+        <v>90.61611310658471</v>
+      </c>
+      <c r="E127" s="2" t="n">
+        <v>24.8</v>
+      </c>
+      <c r="F127" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="G127" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H127" s="2" t="n">
+        <v>42.15010975706134</v>
+      </c>
+      <c r="I127" s="2" t="n">
+        <v>12.37993747398537</v>
+      </c>
+      <c r="J127" s="2" t="n">
+        <v>0.2863272076772039</v>
+      </c>
+      <c r="K127" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L127" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M127" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N127" s="2" t="n">
+        <v>-0.0250700897444002</v>
+      </c>
+      <c r="O127" s="2" t="inlineStr">
+        <is>
+          <t>market_above_ma60, avoid_chase</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="2" t="n">
         <v>6690</v>
       </c>
-      <c r="B127" s="2" t="inlineStr">
+      <c r="B128" s="2" t="inlineStr">
         <is>
           <t>安碁資訊</t>
         </is>
       </c>
-      <c r="C127" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D127" s="2" t="n">
+      <c r="C128" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D128" s="2" t="n">
         <v>81.78146992839007</v>
       </c>
-      <c r="E127" s="2" t="n">
+      <c r="E128" s="2" t="n">
         <v>163.5</v>
       </c>
-      <c r="F127" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-15</t>
-        </is>
-      </c>
-      <c r="G127" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="H127" s="2" t="n">
+      <c r="F128" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="G128" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H128" s="2" t="n">
         <v>40.93053078827083</v>
       </c>
-      <c r="I127" s="2" t="n">
+      <c r="I128" s="2" t="n">
         <v>15.47609072061914</v>
       </c>
-      <c r="J127" s="2" t="n">
+      <c r="J128" s="2" t="n">
         <v>0.4883469975667992</v>
       </c>
-      <c r="K127" s="2" t="n">
+      <c r="K128" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="L127" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M127" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="N127" s="2" t="n">
+      <c r="L128" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M128" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N128" s="2" t="n">
         <v>-0.2901812419519878</v>
       </c>
-      <c r="O127" s="2" t="inlineStr">
+      <c r="O128" s="2" t="inlineStr">
         <is>
           <t>market_above_ma60, avoid_chase</t>
         </is>

</xml_diff>